<commit_message>
Add SQL lessons 1-10 (databases, keys, types, DDL/DML, SELECT, functions, GROUP BY, joins, set operators, subqueries)
All query results are executed against the course database so every
output table is real.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017PtK5YiriwfHtuW98ocpRw
</commit_message>
<xml_diff>
--- a/course/files/excel/excel-09.xlsx
+++ b/course/files/excel/excel-09.xlsx
@@ -26,11 +26,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="0.0000"/>
-    <numFmt numFmtId="166" formatCode="dd-mm-yyyy"/>
-    <numFmt numFmtId="167" formatCode="hh:mm"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="dd-mm-yyyy"/>
+    <numFmt numFmtId="168" formatCode="hh:mm"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -88,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -96,10 +97,11 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -617,20 +619,20 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="12">
         <f>SUM(B2:B5)</f>
         <v/>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="12">
         <f>SUM(C2:C5)</f>
         <v/>
       </c>
-      <c r="D6" s="11">
+      <c r="D6" s="12">
         <f>SUM(D2:D5)</f>
         <v/>
       </c>
@@ -678,7 +680,7 @@
           <t>With GST =Qty*Price*(1+GST_Rate)</t>
         </is>
       </c>
-      <c r="F1" s="12" t="n">
+      <c r="F1" s="13" t="n">
         <v>0.18</v>
       </c>
     </row>
@@ -693,7 +695,7 @@
         <f>A2*B2</f>
         <v/>
       </c>
-      <c r="D2" s="13">
+      <c r="D2" s="14">
         <f>A2*B2*(1+$F$1)</f>
         <v/>
       </c>
@@ -709,7 +711,7 @@
         <f>A3*B3</f>
         <v/>
       </c>
-      <c r="D3" s="13">
+      <c r="D3" s="14">
         <f>A3*B3*(1+$F$1)</f>
         <v/>
       </c>
@@ -725,7 +727,7 @@
         <f>A4*B4</f>
         <v/>
       </c>
-      <c r="D4" s="13">
+      <c r="D4" s="14">
         <f>A4*B4*(1+$F$1)</f>
         <v/>
       </c>
@@ -786,7 +788,7 @@
           <t>12:00</t>
         </is>
       </c>
-      <c r="B3">
+      <c r="B3" s="6">
         <f>TIME(12,0,0)</f>
         <v/>
       </c>
@@ -802,7 +804,7 @@
           <t>06:30</t>
         </is>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="7">
         <f>TIME(6,30,0)</f>
         <v/>
       </c>
@@ -818,7 +820,7 @@
           <t>27-04-2026 18:00</t>
         </is>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="8">
         <f>DATE(2026,4,27)+TIME(18,0,0)</f>
         <v/>
       </c>
@@ -887,7 +889,7 @@
         <f>B2-A2</f>
         <v/>
       </c>
-      <c r="D2" s="8">
+      <c r="D2" s="9">
         <f>A2+30</f>
         <v/>
       </c>
@@ -907,7 +909,7 @@
         <f>B3-A3</f>
         <v/>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="9">
         <f>A3+30</f>
         <v/>
       </c>
@@ -927,7 +929,7 @@
         <f>B4-A4</f>
         <v/>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="9">
         <f>A4+30</f>
         <v/>
       </c>
@@ -1022,15 +1024,15 @@
         <f>WEEKDAY(A2,2)</f>
         <v/>
       </c>
-      <c r="F2" s="8">
+      <c r="F2" s="9">
         <f>EOMONTH(A2,0)</f>
         <v/>
       </c>
-      <c r="G2" s="8">
+      <c r="G2" s="9">
         <f>EOMONTH(A2,-1)+1</f>
         <v/>
       </c>
-      <c r="H2" s="8">
+      <c r="H2" s="9">
         <f>EDATE(A2,3)</f>
         <v/>
       </c>
@@ -1055,15 +1057,15 @@
         <f>WEEKDAY(A3,2)</f>
         <v/>
       </c>
-      <c r="F3" s="8">
+      <c r="F3" s="9">
         <f>EOMONTH(A3,0)</f>
         <v/>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="9">
         <f>EOMONTH(A3,-1)+1</f>
         <v/>
       </c>
-      <c r="H3" s="8">
+      <c r="H3" s="9">
         <f>EDATE(A3,1)</f>
         <v/>
       </c>
@@ -1088,15 +1090,15 @@
         <f>WEEKDAY(A4,2)</f>
         <v/>
       </c>
-      <c r="F4" s="8">
+      <c r="F4" s="9">
         <f>EOMONTH(A4,0)</f>
         <v/>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="9">
         <f>EOMONTH(A4,-1)+1</f>
         <v/>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="9">
         <f>EDATE(A4,12)</f>
         <v/>
       </c>
@@ -1172,7 +1174,7 @@
         <f>NETWORKDAYS(B2,C2,$G$2:$G$4)</f>
         <v/>
       </c>
-      <c r="E2" s="8">
+      <c r="E2" s="9">
         <f>WORKDAY(B2,5,$G$2:$G$4)</f>
         <v/>
       </c>
@@ -1196,7 +1198,7 @@
         <f>NETWORKDAYS(B3,C3,$G$2:$G$4)</f>
         <v/>
       </c>
-      <c r="E3" s="8">
+      <c r="E3" s="9">
         <f>WORKDAY(B3,5,$G$2:$G$4)</f>
         <v/>
       </c>
@@ -1220,7 +1222,7 @@
         <f>NETWORKDAYS.INTL(B4,C4,11,$G$2:$G$4)</f>
         <v/>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="9">
         <f>WORKDAY.INTL(B4,5,11,$G$2:$G$4)</f>
         <v/>
       </c>
@@ -1276,7 +1278,7 @@
           <t>Tenure label</t>
         </is>
       </c>
-      <c r="F1" s="9" t="n">
+      <c r="F1" s="10" t="n">
         <v>46112</v>
       </c>
     </row>
@@ -1517,11 +1519,11 @@
         <f>MOD(A2,100)</f>
         <v/>
       </c>
-      <c r="D2" s="10">
+      <c r="D2" s="11">
         <f>TIME(INT(A2/100),MOD(A2,100),0)</f>
         <v/>
       </c>
-      <c r="E2" s="7">
+      <c r="E2" s="8">
         <f>MOD(D6-D2,1)*24</f>
         <v/>
       </c>
@@ -1538,7 +1540,7 @@
         <f>MOD(A3,100)</f>
         <v/>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="11">
         <f>TIME(INT(A3/100),MOD(A3,100),0)</f>
         <v/>
       </c>
@@ -1555,7 +1557,7 @@
         <f>MOD(A4,100)</f>
         <v/>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="11">
         <f>TIME(INT(A4/100),MOD(A4,100),0)</f>
         <v/>
       </c>
@@ -1572,7 +1574,7 @@
         <f>MOD(A5,100)</f>
         <v/>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="11">
         <f>TIME(INT(A5/100),MOD(A5,100),0)</f>
         <v/>
       </c>
@@ -1589,7 +1591,7 @@
         <f>MOD(A6,100)</f>
         <v/>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="11">
         <f>TIME(INT(A6/100),MOD(A6,100),0)</f>
         <v/>
       </c>

</xml_diff>